<commit_message>
add service staff 2
</commit_message>
<xml_diff>
--- a/exports/KPI_Result_2025_7.xlsx
+++ b/exports/KPI_Result_2025_7.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -481,127 +481,227 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Mai Khanh (MK)</v>
+        <v>Ha Ny (SH)</v>
       </c>
       <c r="B5" t="str">
-        <v>MK</v>
+        <v>SH</v>
       </c>
       <c r="C5" t="str">
-        <v>R&amp;D</v>
+        <v>Sales</v>
       </c>
       <c r="D5">
-        <v>559.9</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>1267.95</v>
+        <v>820.46</v>
       </c>
       <c r="F5" t="str">
-        <v>44.16%</v>
+        <v>0.00%</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Nhiễm (AN)</v>
+        <v>Mai Khanh (MK)</v>
       </c>
       <c r="B6" t="str">
-        <v>AN</v>
+        <v>MK</v>
       </c>
       <c r="C6" t="str">
         <v>R&amp;D</v>
       </c>
       <c r="D6">
-        <v>39.37</v>
+        <v>559.9</v>
       </c>
       <c r="E6">
         <v>1267.95</v>
       </c>
       <c r="F6" t="str">
-        <v>3.11%</v>
+        <v>44.16%</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Nhung (NU)</v>
+        <v>Mai Khanh (MK)</v>
       </c>
       <c r="B7" t="str">
-        <v>NU</v>
+        <v>MK</v>
       </c>
       <c r="C7" t="str">
-        <v>CSM - Bán hàng</v>
+        <v>Sales</v>
       </c>
       <c r="D7">
-        <v>5225.64</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>5628.8</v>
+        <v>820.46</v>
       </c>
       <c r="F7" t="str">
-        <v>92.84%</v>
+        <v>0.00%</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Thiên Hà (HV)</v>
+        <v>Nguyễn Hằng (HN)</v>
       </c>
       <c r="B8" t="str">
-        <v>HV</v>
+        <v>HN</v>
       </c>
       <c r="C8" t="str">
-        <v>CSM - Bán hàng</v>
+        <v>Service Staff</v>
       </c>
       <c r="D8">
-        <v>5225.64</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>5628.8</v>
+        <v>16000</v>
       </c>
       <c r="F8" t="str">
-        <v>92.84%</v>
+        <v>0.00%</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Thành  (BX)</v>
+        <v>Nhiễm (AN)</v>
       </c>
       <c r="B9" t="str">
-        <v>BX</v>
+        <v>AN</v>
       </c>
       <c r="C9" t="str">
         <v>R&amp;D</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>39.37</v>
       </c>
       <c r="E9">
-        <v>1899.48</v>
+        <v>1267.95</v>
       </c>
       <c r="F9" t="str">
-        <v>0.00%</v>
+        <v>3.11%</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Nhiễm (AN)</v>
+      </c>
+      <c r="B10" t="str">
+        <v>AN</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>820.46</v>
+      </c>
+      <c r="F10" t="str">
+        <v>0.00%</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Nhung (NU)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>NU</v>
+      </c>
+      <c r="C11" t="str">
+        <v>CSM - Bán hàng</v>
+      </c>
+      <c r="D11">
+        <v>5225.64</v>
+      </c>
+      <c r="E11">
+        <v>5628.8</v>
+      </c>
+      <c r="F11" t="str">
+        <v>92.84%</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Thao Hong (TA)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>TA</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Service Staff</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>16000</v>
+      </c>
+      <c r="F12" t="str">
+        <v>0.00%</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Thiên Hà (HV)</v>
+      </c>
+      <c r="B13" t="str">
+        <v>HV</v>
+      </c>
+      <c r="C13" t="str">
+        <v>CSM - Bán hàng</v>
+      </c>
+      <c r="D13">
+        <v>5225.64</v>
+      </c>
+      <c r="E13">
+        <v>5628.8</v>
+      </c>
+      <c r="F13" t="str">
+        <v>92.84%</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Thành  (BX)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>BX</v>
+      </c>
+      <c r="C14" t="str">
+        <v>R&amp;D</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>1899.48</v>
+      </c>
+      <c r="F14" t="str">
+        <v>0.00%</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>Truong (XT)</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B15" t="str">
         <v>XT</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C15" t="str">
         <v>Designer</v>
       </c>
-      <c r="D10">
+      <c r="D15">
         <v>2748.07</v>
       </c>
-      <c r="E10">
+      <c r="E15">
         <v>3769.29</v>
       </c>
-      <c r="F10" t="str">
+      <c r="F15" t="str">
         <v>72.91%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>